<commit_message>
Add dihedral, sweep angle. clean code
</commit_message>
<xml_diff>
--- a/Docs/FindusUAV_Plan_A1_QA_TestPlan.xlsx
+++ b/Docs/FindusUAV_Plan_A1_QA_TestPlan.xlsx
@@ -42,13 +42,13 @@
     <t>Test Phase</t>
   </si>
   <si>
-    <t>FindusUAV Configuration - Plan A1 Validation</t>
+    <t>FindusUAV Configuration - Current Validation</t>
   </si>
   <si>
     <t>Objective</t>
   </si>
   <si>
-    <t>Verify UI, boundary validation, and CATIA generation safety for A1 implementation before proceeding to A2.</t>
+    <t>Verify UI, validation, preset storage, and CATIA generation safety for the current implementation before release.</t>
   </si>
   <si>
     <t>Test Suite</t>
@@ -128,7 +128,7 @@
 2. Check numerical and string inputs</t>
   </si>
   <si>
-    <t>Defaults match A1 specs (e.g. Wing Span=3543.65, Wing Airfoil=NACA 4415, Aileron Span=0.40).</t>
+    <t>Defaults match current specs, including sweep=0, dihedral=0, wing airfoil=NACA 4415, aileron span=0.40, and tail cutouts enabled.</t>
   </si>
   <si>
     <t>UI-003</t>
@@ -150,16 +150,16 @@
     <t>UI-004</t>
   </si>
   <si>
-    <t>Deferred Inputs</t>
-  </si>
-  <si>
-    <t>Verify deferred inputs are hidden</t>
-  </si>
-  <si>
-    <t>1. Search UI for Twist, Dihedral, Sweep, Skin Thickness, etc.</t>
-  </si>
-  <si>
-    <t>These high-risk inputs are NOT exposed in the UI.</t>
+    <t>Supported / Deferred Inputs</t>
+  </si>
+  <si>
+    <t>Verify supported inputs are exposed and deferred inputs are hidden</t>
+  </si>
+  <si>
+    <t>1. Search UI for Sweep, Dihedral, Twist, Forward Sweep, Skin Thickness, etc.</t>
+  </si>
+  <si>
+    <t>Swept-back Sweep and Dihedral are exposed with safe ranges. High-risk Twist, Forward Sweep, and Skin Thickness are not exposed.</t>
   </si>
   <si>
     <t>UI-005</t>
@@ -192,7 +192,7 @@
 4. Generate</t>
   </si>
   <si>
-    <t>Validation error surfaces indicating span must be between 500 and 10000 mm. CATIA does not open.</t>
+    <t>Validation error surfaces indicating span must be between 500 and 10000 mm. CATIA generation does not start.</t>
   </si>
   <si>
     <t>W-002</t>
@@ -295,7 +295,7 @@
 4. Generate</t>
   </si>
   <si>
-    <t>Error: Value must be &gt; 0.0 and &lt; 1.0 (recommended 0.15 - 0.60).</t>
+    <t>Error: Aileron span fraction must stay within the supported 0.15 to 0.60 range.</t>
   </si>
   <si>
     <t>T-001</t>
@@ -379,7 +379,7 @@
 3. Trigger Generation</t>
   </si>
   <si>
-    <t>System successfully opens CATIA and generates the EXACT known-good wing and tail geometry with no errors.</t>
+    <t>Wing generation creates a stable CATIA part. Tail generation succeeds when CATIA already has an active PartDocument.</t>
   </si>
   <si>
     <t>E2E-002</t>
@@ -391,13 +391,10 @@
     <t>Verify successful gen with custom valid inputs</t>
   </si>
   <si>
-    <t>1. Set Wing Span = 4000
-2. Set Aileron fraction = 0.35
-3. Set Horiz Half Span = 400
-4. Generate</t>
-  </si>
-  <si>
-    <t>CATIA successfully models the resized UAV. Aileron starts exactly at the wing tip, covering 35% of semi-span.</t>
+    <t>1. Set Wing Span = 4000 / 2. Set Sweep = 12 / 3. Set Dihedral = 3 / 4. Set Aileron fraction = 0.35 / 5. Generate</t>
+  </si>
+  <si>
+    <t>CATIA successfully models the resized swept-back, dihedral wing. Aileron starts at the wing tip and covers 35% of semi-span.</t>
   </si>
   <si>
     <t>E2E-003</t>
@@ -442,13 +439,13 @@
     <t>Verify existing API wrappers</t>
   </si>
   <si>
-    <t>1. Trigger generator via legacy no-argument code entry point</t>
-  </si>
-  <si>
-    <t>Code silently uses default configurations and successfully builds the CATIA model.</t>
-  </si>
-  <si>
-    <t>The Program replace the value with minimum or maximum accepted value instead of throwing error. Still accepted</t>
+    <t>1. Trigger generator through WingGenerationFacade no-argument wrapper</t>
+  </si>
+  <si>
+    <t>Code uses default configurations and successfully builds the CATIA model.</t>
+  </si>
+  <si>
+    <t>Program rejects invalid input with a validation message instead of changing the value silently.</t>
   </si>
   <si>
     <t>Pass</t>

</xml_diff>